<commit_message>
Deployed 7f3b9a6 with MkDocs version: 1.5.3
</commit_message>
<xml_diff>
--- a/Manual/source/CZ/tab/connectors.xlsx
+++ b/Manual/source/CZ/tab/connectors.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="9"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
   </bookViews>
   <sheets>
     <sheet name="X1_24V_5pin_BCZ" sheetId="1" state="visible" r:id="rId2"/>
@@ -18,6 +18,10 @@
     <sheet name="X7_FB2_8pin_BCZ" sheetId="8" state="visible" r:id="rId9"/>
     <sheet name="X3_M1_6pin_BLZP" sheetId="9" state="visible" r:id="rId10"/>
     <sheet name="X4_M2_6pin_BLZP" sheetId="10" state="visible" r:id="rId11"/>
+    <sheet name="X1_24V_5pin_Microlock" sheetId="11" state="visible" r:id="rId12"/>
+    <sheet name="X3_DCbus_2pin_pressfit" sheetId="12" state="visible" r:id="rId13"/>
+    <sheet name="X3_M1_3pin_pressfit" sheetId="13" state="visible" r:id="rId14"/>
+    <sheet name="X4_BR_4pin_Microlock" sheetId="14" state="visible" r:id="rId15"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -29,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="125">
   <si>
     <t xml:space="preserve">Pin č.</t>
   </si>
@@ -398,6 +402,48 @@
   </si>
   <si>
     <t xml:space="preserve">Fáze U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,13 ~ 0,32 mm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Připojení</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">oko M5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+6 ~ +50 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fáze W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fáze V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fáze U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-BR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+BR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-TERM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Tepl. čidla mot.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+TERM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Tepl. čidla mot.</t>
   </si>
 </sst>
 </file>
@@ -515,7 +561,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.38"/>
@@ -623,7 +669,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -735,6 +781,360 @@
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.83"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.83"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
@@ -748,7 +1148,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
@@ -809,7 +1209,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
@@ -1154,7 +1554,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.33"/>
@@ -1247,9 +1647,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.62"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1293,7 +1693,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1502,7 +1902,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1655,7 +2055,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1808,7 +2208,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>

</xml_diff>

<commit_message>
Deployed ce2f689 with MkDocs version: 1.5.3
</commit_message>
<xml_diff>
--- a/Manual/source/CZ/tab/connectors.xlsx
+++ b/Manual/source/CZ/tab/connectors.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="22"/>
   </bookViews>
   <sheets>
     <sheet name="rozcestnik" sheetId="1" state="visible" r:id="rId2"/>
@@ -23,6 +23,14 @@
     <sheet name="X3_DCbus_2pin_pressfit" sheetId="13" state="visible" r:id="rId14"/>
     <sheet name="X3_M1_3pin_pressfit" sheetId="14" state="visible" r:id="rId15"/>
     <sheet name="X4_BR_4pin_Microlock" sheetId="15" state="visible" r:id="rId16"/>
+    <sheet name="X2_DCbus_3pin_wago_2636" sheetId="16" state="visible" r:id="rId17"/>
+    <sheet name="X3_M1_4pin_wago_2626" sheetId="17" state="visible" r:id="rId18"/>
+    <sheet name="X4_M2_4pin_wago_2626" sheetId="18" state="visible" r:id="rId19"/>
+    <sheet name="XBR_BR_6pin_BLF" sheetId="19" state="visible" r:id="rId20"/>
+    <sheet name="X1_24V_5pin_Microfit" sheetId="20" state="visible" r:id="rId21"/>
+    <sheet name="P7_BR_4pin_Microfit" sheetId="21" state="visible" r:id="rId22"/>
+    <sheet name="P8_BR_4pin_Microfit" sheetId="22" state="visible" r:id="rId23"/>
+    <sheet name="P3_Term_2pin_Microfit" sheetId="23" state="visible" r:id="rId24"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -34,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="179">
   <si>
     <t xml:space="preserve">Toto je sešit se zdrojovými tabulkami popisu konektorů TGZ/TGS v češtině. Každý list odpovídá jednomu unikátnímu typu konektoru. Jelikož se často konektory v rámci TGZ opakují (typicky ty na řídicií desce), jsou zde jen jednou. Tj. Např. IO konektor 22pin weidmuller BCZ se používá pořád dokola, je zde tedy zanesen jen jednou jako „X8_IO_22pin_BCZ“</t>
   </si>
@@ -530,13 +538,92 @@
   <si>
     <t xml:space="preserve">+ Tepl. čidla mot.</t>
   </si>
+  <si>
+    <t xml:space="preserve">uzemnění</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,75 ~ 16 mm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,2 ~ 10 mm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-B2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Brzda motor 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,13 ~ 2,5 mm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Brzda motor 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">– Napájení brzdy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Napájení brzdy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Brzda motor 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Brzda motor 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+24V DC napájení řízení</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,05 ~ 0,75 mm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VCC_OUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Výstup +24 VDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+24V DC napájení brzdy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VCCD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+24V DC napájení diag. brzdy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Brzda servomotoru</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Brzda servomotoru</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nezapojuje se</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0V napájení řízení</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TERM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teplotní čidlo PT1000</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -632,7 +719,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -655,6 +742,10 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1594,6 +1685,409 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="str">
+        <f aca="false">+B2</f>
+        <v>-B2</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -1689,6 +2183,372 @@
       </c>
       <c r="D6" s="0" t="s">
         <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.83"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.83"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.83"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.83"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>177</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>178</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>177</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>178</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed d36aae4 with MkDocs version: 1.5.3
</commit_message>
<xml_diff>
--- a/Manual/source/CZ/tab/connectors.xlsx
+++ b/Manual/source/CZ/tab/connectors.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="22"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="25"/>
   </bookViews>
   <sheets>
     <sheet name="rozcestnik" sheetId="1" state="visible" r:id="rId2"/>
@@ -31,6 +31,9 @@
     <sheet name="P7_BR_4pin_Microfit" sheetId="21" state="visible" r:id="rId22"/>
     <sheet name="P8_BR_4pin_Microfit" sheetId="22" state="visible" r:id="rId23"/>
     <sheet name="P3_Term_2pin_Microfit" sheetId="23" state="visible" r:id="rId24"/>
+    <sheet name="X4_M1_6pin_SLS" sheetId="24" state="visible" r:id="rId25"/>
+    <sheet name="X2_PWR_10pin_BLZP" sheetId="25" state="visible" r:id="rId26"/>
+    <sheet name="X2_320_DC_1778078" sheetId="26" state="visible" r:id="rId27"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -42,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="199">
   <si>
     <t xml:space="preserve">Toto je sešit se zdrojovými tabulkami popisu konektorů TGZ/TGS v češtině. Každý list odpovídá jednomu unikátnímu typu konektoru. Jelikož se často konektory v rámci TGZ opakují (typicky ty na řídicií desce), jsou zde jen jednou. Tj. Např. IO konektor 22pin weidmuller BCZ se používá pořád dokola, je zde tedy zanesen jen jednou jako „X8_IO_22pin_BCZ“</t>
   </si>
@@ -615,6 +618,66 @@
   </si>
   <si>
     <t xml:space="preserve">Teplotní čidlo PT1000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,2 ~ 2,5 mm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Střední pracovní vodič</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fáze </t>
+  </si>
+  <si>
+    <t xml:space="preserve">+RB </t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Brzdný odpor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-RB </t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Brzdný odpor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+DC </t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Napájení meziobvodu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-DC </t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Napájení meziobvodu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">T+ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Termistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T- </t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Termistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+140 ~ +320V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max. 6 mm2</t>
   </si>
 </sst>
 </file>
@@ -724,16 +787,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -746,6 +805,10 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -826,9 +889,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultColWidth="12.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.81"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="31.81"/>
   </cols>
@@ -975,7 +1038,7 @@
       <c r="G11" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="H11" s="3" t="s">
         <v>17</v>
       </c>
     </row>
@@ -988,7 +1051,7 @@
       <c r="G12" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="3" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1001,7 +1064,7 @@
       <c r="G13" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="H13" s="3" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1014,7 +1077,7 @@
       <c r="G14" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H14" s="3" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1027,7 +1090,7 @@
       <c r="G15" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="H15" s="3" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1040,7 +1103,7 @@
       <c r="G16" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="3" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1087,7 +1150,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1193,7 +1256,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="5"/>
+      <c r="C18" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1212,7 +1275,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1318,7 +1381,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="5"/>
+      <c r="C18" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1337,7 +1400,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.38"/>
@@ -1445,7 +1508,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1495,7 +1558,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="5"/>
+      <c r="C18" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1514,7 +1577,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1578,7 +1641,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="5"/>
+      <c r="C18" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1597,7 +1660,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.38"/>
@@ -1691,7 +1754,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1755,7 +1818,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="5"/>
+      <c r="C18" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1774,7 +1837,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1852,7 +1915,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="5"/>
+      <c r="C18" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1871,7 +1934,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1949,7 +2012,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="5"/>
+      <c r="C18" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1968,7 +2031,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27.23"/>
@@ -1993,7 +2056,7 @@
       <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>156</v>
       </c>
       <c r="C2" s="0" t="s">
@@ -2050,7 +2113,7 @@
       <c r="A6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>162</v>
       </c>
       <c r="C6" s="0" t="s">
@@ -2064,7 +2127,7 @@
       <c r="A7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>164</v>
       </c>
       <c r="C7" s="0" t="s">
@@ -2075,7 +2138,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="5"/>
+      <c r="C18" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2094,7 +2157,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.38"/>
@@ -2202,11 +2265,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.83"/>
   </cols>
   <sheetData>
@@ -2311,7 +2374,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
@@ -2406,7 +2469,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
@@ -2501,7 +2564,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
@@ -2549,6 +2612,390 @@
       </c>
       <c r="D3" s="0" t="s">
         <v>167</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="4"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="4"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.1"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>197</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -2568,7 +3015,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
@@ -2629,7 +3076,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
@@ -2974,7 +3421,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.33"/>
@@ -3067,7 +3514,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.62"/>
   </cols>
@@ -3113,7 +3560,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -3303,7 +3750,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="5"/>
+      <c r="C18" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3322,7 +3769,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -3456,7 +3903,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="5"/>
+      <c r="C18" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3475,7 +3922,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -3609,7 +4056,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="5"/>
+      <c r="C18" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Deployed c445a28 with MkDocs version: 1.5.3
</commit_message>
<xml_diff>
--- a/Manual/source/CZ/tab/connectors.xlsx
+++ b/Manual/source/CZ/tab/connectors.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="25"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="27"/>
   </bookViews>
   <sheets>
     <sheet name="rozcestnik" sheetId="1" state="visible" r:id="rId2"/>
@@ -34,6 +34,8 @@
     <sheet name="X4_M1_6pin_SLS" sheetId="24" state="visible" r:id="rId25"/>
     <sheet name="X2_PWR_10pin_BLZP" sheetId="25" state="visible" r:id="rId26"/>
     <sheet name="X2_320_DC_1778078" sheetId="26" state="visible" r:id="rId27"/>
+    <sheet name="X4_M1_6pin_BLF" sheetId="27" state="visible" r:id="rId28"/>
+    <sheet name="X2_PWR_12pin_BLZ" sheetId="28" state="visible" r:id="rId29"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -45,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="214">
   <si>
     <t xml:space="preserve">Toto je sešit se zdrojovými tabulkami popisu konektorů TGZ/TGS v češtině. Každý list odpovídá jednomu unikátnímu typu konektoru. Jelikož se často konektory v rámci TGZ opakují (typicky ty na řídicií desce), jsou zde jen jednou. Tj. Např. IO konektor 22pin weidmuller BCZ se používá pořád dokola, je zde tedy zanesen jen jednou jako „X8_IO_22pin_BCZ“</t>
   </si>
@@ -678,6 +680,51 @@
   </si>
   <si>
     <t xml:space="preserve">Max. 6 mm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,5 ~ 2,5 mm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fáze 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fáze 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L3 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fáze 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RBin </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brzdný odpor interní</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEL </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volba brzdného odporu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RBex </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brzdný odpor externí</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+Termistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Termistor</t>
   </si>
 </sst>
 </file>
@@ -889,9 +936,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultColWidth="12.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="31.81"/>
   </cols>
@@ -1150,7 +1197,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1275,7 +1322,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1400,7 +1447,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.38"/>
@@ -1508,7 +1555,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1577,7 +1624,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1660,7 +1707,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.38"/>
@@ -1754,7 +1801,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1837,7 +1884,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -1934,7 +1981,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -2031,7 +2078,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27.23"/>
@@ -2157,7 +2204,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.38"/>
@@ -2265,7 +2312,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
@@ -2374,7 +2421,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
@@ -2469,7 +2516,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
@@ -2564,7 +2611,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
@@ -2631,7 +2678,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -2756,7 +2803,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.79"/>
@@ -2937,7 +2984,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.1"/>
   </cols>
@@ -2996,6 +3043,337 @@
       </c>
       <c r="D4" s="0" t="s">
         <v>198</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="4"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>200</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>203</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>204</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>210</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>211</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>188</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>190</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>191</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>212</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>195</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -3015,7 +3393,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
@@ -3076,7 +3454,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
@@ -3421,7 +3799,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.33"/>
@@ -3514,7 +3892,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.62"/>
   </cols>
@@ -3560,7 +3938,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -3769,7 +4147,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
@@ -3922,7 +4300,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>

</xml_diff>

<commit_message>
Deployed 1f236b5 with MkDocs version: 1.5.3
</commit_message>
<xml_diff>
--- a/Manual/source/CZ/tab/connectors.xlsx
+++ b/Manual/source/CZ/tab/connectors.xlsx
@@ -5,37 +5,39 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="27"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="29"/>
   </bookViews>
   <sheets>
-    <sheet name="rozcestnik" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="X1_24V_5pin_BCZ" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="X2_48_DC_1778065" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="X8_IO_22pin_BCZ" sheetId="4" state="visible" r:id="rId5"/>
-    <sheet name="X10_CAN_4pin_BCZ" sheetId="5" state="visible" r:id="rId6"/>
-    <sheet name="LEDsigAx12" sheetId="6" state="visible" r:id="rId7"/>
-    <sheet name="X5_FBE_12pin_BCZ" sheetId="7" state="visible" r:id="rId8"/>
-    <sheet name="X6_FB1_8pin_BCZ" sheetId="8" state="visible" r:id="rId9"/>
-    <sheet name="X7_FB2_8pin_BCZ" sheetId="9" state="visible" r:id="rId10"/>
-    <sheet name="X3_M1_6pin_BLZP" sheetId="10" state="visible" r:id="rId11"/>
-    <sheet name="X4_M2_6pin_BLZP" sheetId="11" state="visible" r:id="rId12"/>
-    <sheet name="X1_24V_5pin_Microlock" sheetId="12" state="visible" r:id="rId13"/>
-    <sheet name="X3_DCbus_2pin_pressfit" sheetId="13" state="visible" r:id="rId14"/>
-    <sheet name="X3_M1_3pin_pressfit" sheetId="14" state="visible" r:id="rId15"/>
-    <sheet name="X4_BR_4pin_Microlock" sheetId="15" state="visible" r:id="rId16"/>
-    <sheet name="X2_DCbus_3pin_wago_2636" sheetId="16" state="visible" r:id="rId17"/>
-    <sheet name="X3_M1_4pin_wago_2626" sheetId="17" state="visible" r:id="rId18"/>
-    <sheet name="X4_M2_4pin_wago_2626" sheetId="18" state="visible" r:id="rId19"/>
-    <sheet name="XBR_BR_6pin_BLF" sheetId="19" state="visible" r:id="rId20"/>
-    <sheet name="X1_24V_5pin_Microfit" sheetId="20" state="visible" r:id="rId21"/>
-    <sheet name="P7_BR_4pin_Microfit" sheetId="21" state="visible" r:id="rId22"/>
-    <sheet name="P8_BR_4pin_Microfit" sheetId="22" state="visible" r:id="rId23"/>
-    <sheet name="P3_Term_2pin_Microfit" sheetId="23" state="visible" r:id="rId24"/>
-    <sheet name="X4_M1_6pin_SLS" sheetId="24" state="visible" r:id="rId25"/>
-    <sheet name="X2_PWR_10pin_BLZP" sheetId="25" state="visible" r:id="rId26"/>
-    <sheet name="X2_320_DC_1778078" sheetId="26" state="visible" r:id="rId27"/>
-    <sheet name="X4_M1_6pin_BLF" sheetId="27" state="visible" r:id="rId28"/>
-    <sheet name="X2_PWR_12pin_BLZ" sheetId="28" state="visible" r:id="rId29"/>
+    <sheet name="rozcestnik" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="X1_24V_5pin_BCZ" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="X2_48_DC_1778065" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="X8_IO_22pin_BCZ" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="X10_CAN_4pin_BCZ" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="LEDsigAx12" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="X5_FBE_12pin_BCZ" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="X6_FB1_8pin_BCZ" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="X7_FB2_8pin_BCZ" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="X3_M1_6pin_BLZP" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="X4_M2_6pin_BLZP" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="X1_24V_5pin_Microlock" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="X3_DCbus_2pin_pressfit" sheetId="13" state="visible" r:id="rId15"/>
+    <sheet name="X3_M1_3pin_pressfit" sheetId="14" state="visible" r:id="rId16"/>
+    <sheet name="X4_BR_4pin_Microlock" sheetId="15" state="visible" r:id="rId17"/>
+    <sheet name="X2_DCbus_3pin_wago_2636" sheetId="16" state="visible" r:id="rId18"/>
+    <sheet name="X3_M1_4pin_wago_2626" sheetId="17" state="visible" r:id="rId19"/>
+    <sheet name="X4_M2_4pin_wago_2626" sheetId="18" state="visible" r:id="rId20"/>
+    <sheet name="XBR_BR_6pin_BLF" sheetId="19" state="visible" r:id="rId21"/>
+    <sheet name="X1_24V_5pin_Microfit" sheetId="20" state="visible" r:id="rId22"/>
+    <sheet name="P7_BR_4pin_Microfit" sheetId="21" state="visible" r:id="rId23"/>
+    <sheet name="P8_BR_4pin_Microfit" sheetId="22" state="visible" r:id="rId24"/>
+    <sheet name="P3_Term_2pin_Microfit" sheetId="23" state="visible" r:id="rId25"/>
+    <sheet name="X4_M1_6pin_SLS" sheetId="24" state="visible" r:id="rId26"/>
+    <sheet name="X2_PWR_10pin_BLZP" sheetId="25" state="visible" r:id="rId27"/>
+    <sheet name="X2_320_DC_1778078" sheetId="26" state="visible" r:id="rId28"/>
+    <sheet name="X4_M1_6pin_BLF" sheetId="27" state="visible" r:id="rId29"/>
+    <sheet name="X2_PWR_12pin_BLZ" sheetId="28" state="visible" r:id="rId30"/>
+    <sheet name="X2_D560DCbus" sheetId="29" state="visible" r:id="rId31"/>
+    <sheet name="X3_M1_4pin_wago_2636" sheetId="30" state="visible" r:id="rId32"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -47,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="219">
   <si>
     <t xml:space="preserve">Toto je sešit se zdrojovými tabulkami popisu konektorů TGZ/TGS v češtině. Každý list odpovídá jednomu unikátnímu typu konektoru. Jelikož se často konektory v rámci TGZ opakují (typicky ty na řídicií desce), jsou zde jen jednou. Tj. Např. IO konektor 22pin weidmuller BCZ se používá pořád dokola, je zde tedy zanesen jen jednou jako „X8_IO_22pin_BCZ“</t>
   </si>
@@ -725,6 +727,21 @@
   </si>
   <si>
     <t xml:space="preserve">-Termistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-DC IN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ DC bus vstup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dle oka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+DC IN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- DC bus vstup</t>
   </si>
 </sst>
 </file>
@@ -829,32 +846,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -930,238 +951,344 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultColWidth="12.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="31.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="31.81"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="F8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G8" s="0" t="s">
+      <c r="G8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H8" s="0" t="s">
+      <c r="H8" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="1" t="n">
         <v>48</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="0" t="n">
+      <c r="D10" s="1" t="n">
         <v>48</v>
       </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="0" t="s">
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="0" t="n">
+      <c r="D11" s="1" t="n">
         <v>48</v>
       </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="0" t="s">
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H11" s="4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D12" s="0" t="n">
+      <c r="D12" s="1" t="n">
         <v>48</v>
       </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="0" t="s">
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D13" s="0" t="n">
+      <c r="D13" s="1" t="n">
         <v>48</v>
       </c>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="0" t="s">
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="H13" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D14" s="0" t="n">
+      <c r="D14" s="1" t="n">
         <v>48</v>
       </c>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="0" t="s">
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="H14" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D15" s="0" t="n">
+      <c r="D15" s="1" t="n">
         <v>48</v>
       </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="0" t="s">
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="H15" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D16" s="0" t="n">
+      <c r="D16" s="1" t="n">
         <v>48</v>
       </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="0" t="s">
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="H16" s="4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D17" s="0" t="n">
+      <c r="D17" s="1" t="n">
         <v>48</v>
       </c>
-      <c r="E17" s="0" t="n">
+      <c r="E17" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="F17" s="0" t="n">
+      <c r="F17" s="1" t="n">
         <v>250</v>
       </c>
     </row>
@@ -1192,118 +1319,118 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1317,118 +1444,118 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1442,99 +1569,99 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>139</v>
       </c>
     </row>
@@ -1550,62 +1677,62 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1619,76 +1746,76 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1702,85 +1829,85 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>139</v>
       </c>
     </row>
@@ -1796,76 +1923,76 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1879,90 +2006,90 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1976,90 +2103,90 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2073,119 +2200,119 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="27.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="str">
+      <c r="B3" s="1" t="str">
         <f aca="false">+B2</f>
         <v>-B2</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2199,99 +2326,99 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2307,100 +2434,100 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>167</v>
       </c>
     </row>
@@ -2416,86 +2543,86 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>167</v>
       </c>
     </row>
@@ -2511,86 +2638,86 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>167</v>
       </c>
     </row>
@@ -2606,58 +2733,58 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>167</v>
       </c>
     </row>
@@ -2673,118 +2800,118 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2798,174 +2925,174 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="7" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="n">
+      <c r="A2" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2979,69 +3106,69 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.1"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>198</v>
       </c>
     </row>
@@ -3057,118 +3184,118 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3182,199 +3309,295 @@
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
+      <c r="A13" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" s="1" t="s">
         <v>128</v>
       </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3388,7 +3611,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -3396,46 +3619,143 @@
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>45</v>
       </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3449,336 +3769,336 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D23"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
+      <c r="A13" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="n">
+      <c r="A14" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="n">
+      <c r="A15" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="n">
+      <c r="A16" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="n">
+      <c r="A17" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="n">
+      <c r="A18" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D18" s="0" t="s">
+      <c r="D18" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="n">
+      <c r="A19" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D19" s="0" t="s">
+      <c r="D19" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="n">
+      <c r="A20" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="D20" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="n">
+      <c r="A21" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D21" s="0" t="s">
+      <c r="D21" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="n">
+      <c r="A22" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D22" s="0" t="s">
+      <c r="D22" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="n">
+      <c r="A23" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="C23" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D23" s="0" t="s">
+      <c r="D23" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -3794,84 +4114,84 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -3887,37 +4207,37 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.62"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>102</v>
       </c>
     </row>
@@ -3933,202 +4253,202 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
+      <c r="A13" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" s="1" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4142,146 +4462,146 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4295,146 +4615,146 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="4"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Deployed b5c04f2 with MkDocs version: 1.5.3
</commit_message>
<xml_diff>
--- a/Manual/source/CZ/tab/connectors.xlsx
+++ b/Manual/source/CZ/tab/connectors.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="29"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="35"/>
   </bookViews>
   <sheets>
     <sheet name="rozcestnik" sheetId="1" state="visible" r:id="rId3"/>
@@ -38,6 +38,12 @@
     <sheet name="X2_PWR_12pin_BLZ" sheetId="28" state="visible" r:id="rId30"/>
     <sheet name="X2_D560DCbus" sheetId="29" state="visible" r:id="rId31"/>
     <sheet name="X3_M1_4pin_wago_2636" sheetId="30" state="visible" r:id="rId32"/>
+    <sheet name="X4_M2_4pin_wago_2636" sheetId="31" state="visible" r:id="rId33"/>
+    <sheet name="X14_BR1_4pin_LSF" sheetId="32" state="visible" r:id="rId34"/>
+    <sheet name="X15_BR2_4pin_LSF" sheetId="33" state="visible" r:id="rId35"/>
+    <sheet name="X1_ACIN_PC5" sheetId="34" state="visible" r:id="rId36"/>
+    <sheet name="X2_DC_8pin_PC5" sheetId="35" state="visible" r:id="rId37"/>
+    <sheet name="X3_DO_4pin_BCZ" sheetId="36" state="visible" r:id="rId38"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -49,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="243">
   <si>
     <t xml:space="preserve">Toto je sešit se zdrojovými tabulkami popisu konektorů TGZ/TGS v češtině. Každý list odpovídá jednomu unikátnímu typu konektoru. Jelikož se často konektory v rámci TGZ opakují (typicky ty na řídicií desce), jsou zde jen jednou. Tj. Např. IO konektor 22pin weidmuller BCZ se používá pořád dokola, je zde tedy zanesen jen jednou jako „X8_IO_22pin_BCZ“</t>
   </si>
@@ -723,9 +729,15 @@
     <t xml:space="preserve">Brzdný odpor externí</t>
   </si>
   <si>
+    <t xml:space="preserve">T+</t>
+  </si>
+  <si>
     <t xml:space="preserve">+Termistor</t>
   </si>
   <si>
+    <t xml:space="preserve">T-</t>
+  </si>
+  <si>
     <t xml:space="preserve">-Termistor</t>
   </si>
   <si>
@@ -742,6 +754,72 @@
   </si>
   <si>
     <t xml:space="preserve">- DC bus vstup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Brzda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,13 ~ 1,5 mm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Brzda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fáze</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  + DC </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - DC </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  PE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  SEL </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  + RB </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - RB </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  + T </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - T </t>
+  </si>
+  <si>
+    <t xml:space="preserve">RDY1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signál „Ready“ kontakt 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RDY2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signál „Ready“ kontakt 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERR1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signál „Error“ kontakt 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERR2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signál „Error“ kontakt 2</t>
   </si>
 </sst>
 </file>
@@ -3480,10 +3558,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>128</v>
@@ -3494,10 +3572,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>195</v>
+        <v>214</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>128</v>
@@ -3546,13 +3624,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3560,13 +3638,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>218</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3703,10 +3781,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>154</v>
@@ -3717,10 +3795,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>154</v>
@@ -3731,10 +3809,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>154</v>
@@ -3745,17 +3823,785 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>154</v>
       </c>
     </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="0"/>
+      <c r="C14" s="0"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="0"/>
+      <c r="C15" s="0"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="0"/>
+      <c r="C16" s="0"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="0"/>
+      <c r="C17" s="0"/>
+    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C18" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="0"/>
+      <c r="C14" s="0"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="0"/>
+      <c r="C15" s="0"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="0"/>
+      <c r="C16" s="0"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="0"/>
+      <c r="C17" s="0"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="0"/>
+      <c r="C10" s="0"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="0"/>
+      <c r="C14" s="0"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="0"/>
+      <c r="C15" s="0"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="0"/>
+      <c r="C16" s="0"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="0"/>
+      <c r="C17" s="0"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="0"/>
+      <c r="C10" s="0"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="0"/>
+      <c r="C14" s="0"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="0"/>
+      <c r="C15" s="0"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="0"/>
+      <c r="C16" s="0"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="0"/>
+      <c r="C17" s="0"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.79"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.72"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>191</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>231</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>185</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>187</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>194</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>234</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>196</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="0"/>
+      <c r="C13" s="0"/>
+      <c r="D13" s="0"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="0"/>
+      <c r="C14" s="0"/>
+      <c r="D14" s="0"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="0"/>
+      <c r="C15" s="0"/>
+      <c r="D15" s="0"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="0"/>
+      <c r="C16" s="0"/>
+      <c r="D16" s="0"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="0"/>
+      <c r="C17" s="0"/>
+      <c r="D17" s="0"/>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="0"/>
+      <c r="C18" s="0"/>
+      <c r="D18" s="0"/>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="0"/>
+      <c r="C19" s="0"/>
+      <c r="D19" s="0"/>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="0"/>
+      <c r="C20" s="0"/>
+      <c r="D20" s="0"/>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="0"/>
+      <c r="C21" s="0"/>
+      <c r="D21" s="0"/>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="0"/>
+      <c r="C22" s="0"/>
+      <c r="D22" s="0"/>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="0"/>
+      <c r="C23" s="0"/>
+      <c r="D23" s="0"/>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="0"/>
+      <c r="C24" s="0"/>
+      <c r="D24" s="0"/>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="0"/>
+      <c r="C25" s="0"/>
+      <c r="D25" s="0"/>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="0"/>
+      <c r="C26" s="0"/>
+      <c r="D26" s="0"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.83"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>34</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Deployed 48399a7 with MkDocs version: 1.5.3
</commit_message>
<xml_diff>
--- a/Manual/source/CZ/tab/connectors.xlsx
+++ b/Manual/source/CZ/tab/connectors.xlsx
@@ -5,18 +5,18 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="35"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="38"/>
   </bookViews>
   <sheets>
     <sheet name="rozcestnik" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="X1_24V_5pin_BCZ" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="X2_48_DC_1778065" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="X8_IO_22pin_BCZ" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="X10_CAN_4pin_BCZ" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="X8_IO_22pin_B2CF" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="X10_CAN_4pin_B2CF" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="LEDsigAx12" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="X5_FBE_12pin_BCZ" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="X6_FB1_8pin_BCZ" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="X7_FB2_8pin_BCZ" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="X5_FBE_12pin_B2CF" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="X6_FB1_8pin_B2CF" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="X7_FB2_8pin_B2CF" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="X3_M1_6pin_BLZP" sheetId="10" state="visible" r:id="rId12"/>
     <sheet name="X4_M2_6pin_BLZP" sheetId="11" state="visible" r:id="rId13"/>
     <sheet name="X1_24V_5pin_Microlock" sheetId="12" state="visible" r:id="rId14"/>
@@ -44,6 +44,10 @@
     <sheet name="X1_ACIN_PC5" sheetId="34" state="visible" r:id="rId36"/>
     <sheet name="X2_DC_8pin_PC5" sheetId="35" state="visible" r:id="rId37"/>
     <sheet name="X3_DO_4pin_BCZ" sheetId="36" state="visible" r:id="rId38"/>
+    <sheet name="X3_24V_BLF_2_5" sheetId="37" state="visible" r:id="rId39"/>
+    <sheet name="X5_DI_10pin_B2CF" sheetId="38" state="visible" r:id="rId40"/>
+    <sheet name="X10_DO_10pin_B2CF" sheetId="39" state="visible" r:id="rId41"/>
+    <sheet name="S1_SWITCH_CAN" sheetId="40" state="visible" r:id="rId42"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -55,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="280">
   <si>
     <t xml:space="preserve">Toto je sešit se zdrojovými tabulkami popisu konektorů TGZ/TGS v češtině. Každý list odpovídá jednomu unikátnímu typu konektoru. Jelikož se často konektory v rámci TGZ opakují (typicky ty na řídicií desce), jsou zde jen jednou. Tj. Např. IO konektor 22pin weidmuller BCZ se používá pořád dokola, je zde tedy zanesen jen jednou jako „X8_IO_22pin_BCZ“</t>
   </si>
@@ -820,6 +824,117 @@
   </si>
   <si>
     <t xml:space="preserve">Signál „Error“ kontakt 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+PWR 24V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vstup pro napájecí napětí 24V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,08 ~ 0,5 mm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PWRCOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vstup pro napájecí zem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Digitální vstup č. 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Digitální vstup č. 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUTCOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Společná zem DO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUTPWR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Společné napájení DO 24V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pozice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funkce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nahoře</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vypnuto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAN není terminován</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zapnuto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAN je terminován</t>
   </si>
 </sst>
 </file>
@@ -3832,22 +3947,6 @@
         <v>154</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0"/>
-      <c r="C14" s="0"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0"/>
-      <c r="C15" s="0"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0"/>
-      <c r="C16" s="0"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0"/>
-      <c r="C17" s="0"/>
-    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C18" s="5"/>
     </row>
@@ -3945,22 +4044,6 @@
         <v>154</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0"/>
-      <c r="C14" s="0"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0"/>
-      <c r="C15" s="0"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0"/>
-      <c r="C16" s="0"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0"/>
-      <c r="C17" s="0"/>
-    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C18" s="5"/>
     </row>
@@ -4058,26 +4141,6 @@
         <v>222</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0"/>
-      <c r="C10" s="0"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0"/>
-      <c r="C14" s="0"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0"/>
-      <c r="C15" s="0"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0"/>
-      <c r="C16" s="0"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0"/>
-      <c r="C17" s="0"/>
-    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C18" s="5"/>
     </row>
@@ -4175,26 +4238,6 @@
         <v>222</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0"/>
-      <c r="C10" s="0"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0"/>
-      <c r="C14" s="0"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0"/>
-      <c r="C15" s="0"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0"/>
-      <c r="C16" s="0"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0"/>
-      <c r="C17" s="0"/>
-    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C18" s="5"/>
     </row>
@@ -4217,7 +4260,7 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="19.79"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4263,13 +4306,13 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>226</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -4292,7 +4335,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
@@ -4301,128 +4344,128 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>198</v>
       </c>
     </row>
@@ -4437,76 +4480,6 @@
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="0"/>
-      <c r="C13" s="0"/>
-      <c r="D13" s="0"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0"/>
-      <c r="C14" s="0"/>
-      <c r="D14" s="0"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0"/>
-      <c r="C15" s="0"/>
-      <c r="D15" s="0"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0"/>
-      <c r="C16" s="0"/>
-      <c r="D16" s="0"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0"/>
-      <c r="C17" s="0"/>
-      <c r="D17" s="0"/>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="0"/>
-      <c r="C18" s="0"/>
-      <c r="D18" s="0"/>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0"/>
-      <c r="C19" s="0"/>
-      <c r="D19" s="0"/>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="0"/>
-      <c r="C20" s="0"/>
-      <c r="D20" s="0"/>
-    </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="0"/>
-      <c r="C21" s="0"/>
-      <c r="D21" s="0"/>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="0"/>
-      <c r="C22" s="0"/>
-      <c r="D22" s="0"/>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="0"/>
-      <c r="C23" s="0"/>
-      <c r="D23" s="0"/>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="0"/>
-      <c r="C24" s="0"/>
-      <c r="D24" s="0"/>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="0"/>
-      <c r="C25" s="0"/>
-      <c r="D25" s="0"/>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="0"/>
-      <c r="C26" s="0"/>
-      <c r="D26" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4614,6 +4587,409 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.83"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -4947,6 +5323,96 @@
       <c r="D23" s="1" t="s">
         <v>50</v>
       </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Deployed f3213c7 with MkDocs version: 1.5.3
</commit_message>
<xml_diff>
--- a/Manual/source/CZ/tab/connectors.xlsx
+++ b/Manual/source/CZ/tab/connectors.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="38"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="43"/>
   </bookViews>
   <sheets>
     <sheet name="rozcestnik" sheetId="1" state="visible" r:id="rId3"/>
@@ -48,6 +48,10 @@
     <sheet name="X5_DI_10pin_B2CF" sheetId="38" state="visible" r:id="rId40"/>
     <sheet name="X10_DO_10pin_B2CF" sheetId="39" state="visible" r:id="rId41"/>
     <sheet name="S1_SWITCH_CAN" sheetId="40" state="visible" r:id="rId42"/>
+    <sheet name="X1_24V_5pin_BCZ_TGM" sheetId="41" state="visible" r:id="rId43"/>
+    <sheet name="X5_FBE_12pin_B2CF_TGM" sheetId="42" state="visible" r:id="rId44"/>
+    <sheet name="X6_FB1_8pin_B2CF_TGM" sheetId="43" state="visible" r:id="rId45"/>
+    <sheet name="X7_FB2_8pin_B2CF_TGM" sheetId="44" state="visible" r:id="rId46"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -59,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="286">
   <si>
     <t xml:space="preserve">Toto je sešit se zdrojovými tabulkami popisu konektorů TGZ/TGS v češtině. Každý list odpovídá jednomu unikátnímu typu konektoru. Jelikož se často konektory v rámci TGZ opakují (typicky ty na řídicií desce), jsou zde jen jednou. Tj. Např. IO konektor 22pin weidmuller BCZ se používá pořád dokola, je zde tedy zanesen jen jednou jako „X8_IO_22pin_BCZ“</t>
   </si>
@@ -935,6 +939,24 @@
   </si>
   <si>
     <t xml:space="preserve">CAN je terminován</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EI1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozšířený vstup 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EI2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozšířený vstup 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+24V napájení</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSI</t>
   </si>
 </sst>
 </file>
@@ -4692,7 +4714,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4846,7 +4868,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5345,74 +5367,561 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="18.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.83"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="0" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>272</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>273</v>
+        <v>103</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>274</v>
+      <c r="A2" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>275</v>
+        <v>109</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>276</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>277</v>
+      <c r="A3" s="1" t="n">
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>278</v>
+        <v>109</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>279</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1"/>
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1"/>
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1"/>
+      <c r="A6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1"/>
+      <c r="A7" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1"/>
+      <c r="A8" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1"/>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1"/>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1"/>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1"/>
+      <c r="A9" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C18" s="5"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Deployed 3426d3fe with MkDocs version: 1.5.3
</commit_message>
<xml_diff>
--- a/Manual/source/CZ/tab/connectors.xlsx
+++ b/Manual/source/CZ/tab/connectors.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="52"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="17"/>
   </bookViews>
   <sheets>
     <sheet name="rozcestnik" sheetId="1" state="visible" r:id="rId3"/>
@@ -791,7 +791,7 @@
     <t xml:space="preserve">0,75 ~ 16 mm2</t>
   </si>
   <si>
-    <t xml:space="preserve">0,2 ~ 10 mm2</t>
+    <t xml:space="preserve">0,2 ~ 6 mm2</t>
   </si>
   <si>
     <t xml:space="preserve">-B2</t>
@@ -12127,152 +12127,112 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="49.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>400</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>400</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>406</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>408</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0"/>
-      <c r="C10" s="0"/>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="0"/>
-      <c r="C11" s="0"/>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="0"/>
-      <c r="C12" s="0"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="0"/>
-      <c r="C13" s="0"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0"/>
-      <c r="C14" s="0"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0"/>
-      <c r="C15" s="0"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0"/>
-      <c r="C16" s="0"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0"/>
-      <c r="C17" s="0"/>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="0"/>
-      <c r="C18" s="0"/>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0"/>
-      <c r="C19" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -12295,7 +12255,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12316,7 +12276,7 @@
       <c r="B2" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>410</v>
       </c>
     </row>
@@ -12327,7 +12287,7 @@
       <c r="B3" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>412</v>
       </c>
     </row>
@@ -12338,7 +12298,7 @@
       <c r="B4" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>413</v>
       </c>
     </row>
@@ -12349,7 +12309,7 @@
       <c r="B5" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>414</v>
       </c>
     </row>
@@ -12360,7 +12320,7 @@
       <c r="B6" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>416</v>
       </c>
     </row>
@@ -12371,7 +12331,7 @@
       <c r="B7" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>417</v>
       </c>
     </row>
@@ -12382,7 +12342,7 @@
       <c r="B8" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>418</v>
       </c>
     </row>
@@ -12393,7 +12353,7 @@
       <c r="B9" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>419</v>
       </c>
     </row>
@@ -12404,7 +12364,7 @@
       <c r="B10" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>420</v>
       </c>
     </row>
@@ -12415,7 +12375,7 @@
       <c r="B11" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>421</v>
       </c>
     </row>
@@ -12449,115 +12409,113 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="29.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>423</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>425</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>427</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>429</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>431</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>433</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>435</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>437</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
-      <c r="C10" s="0"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
-      <c r="C11" s="0"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>

</xml_diff>